<commit_message>
Add wheel AliExpress cart list with specific listings
- New DAZ_wheel_AliExpress_cart_list_AUD.xlsx: one line per cart item
  with the exact listing, the option to pick, a target price and an
  alternative link. Yellow "your cart price" cells plus an "over target
  by" column show which lines push the cart past the AUD 191 target. A
  "don't add these" block covers the usual culprits: FANAUE clamp, suede
  rim, buttons upgrade, per-seller shipping.
- Wheel list (and the combined list) now point at the same specific
  listings: DAZ's pulley/belt/idler listings, an AU-plug 24 V adapter,
  an AMASS XT60 pack, a cheap Arca-Swiss clamp and a resistor pack.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEYLvGWigrKvVwvVek2yBU
</commit_message>
<xml_diff>
--- a/parts-lists/DAZ_all_three_best_value_parts_list_AUD.xlsx
+++ b/parts-lists/DAZ_all_three_best_value_parts_list_AUD.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="365">
   <si>
     <t xml:space="preserve">DAZ wheel + shifter + pedals – best-value parts list for all three (AUD)</t>
   </si>
@@ -151,166 +151,181 @@
     <t xml:space="preserve">GT2 timing pulley, 20T, 6 mm bore, 6 mm belt</t>
   </si>
   <si>
+    <t xml:space="preserve">Kept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: GT2 20T 6 mm bore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard part – any seller with these sizes. Goes on the encoder shaft.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 search: GT2 20T pulleys from US$0.79 (bore varies) – about US$1 for 6 mm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GT2 closed-loop belt, 212 mm, 6 mm wide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: GT2 belt 212 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must be a closed loop, 212 mm long, 6 mm wide.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 search: 6 mm GT2 loops from US$3.04 (US store).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GT2 idler, 20T toothed, 5 mm bore, 6 mm wide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: GT2 idler 20T 5 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keeps the encoder belt tight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAZ's link: US$2.24 (May 2025) ≈ AUD 3.55 incl. GST.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power supply, 24 V 10 A (240 W), AU plug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheaper – AU-plug adapter listing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress: 24 V adapter (pick 10A, AU plug)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 24V 10A power supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The full 240 W gives the full force. Pick an enclosed 'adapter' type with an AU plug, so there's no 240 V wiring to do. Any brand works.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAZ's link: US$11.15 (May 2025) ≈ AUD 18 incl. GST. 2026 search: 24 V 10 A adapters with AU plug ≈ US$19 (US store) ≈ AUD 30 incl. GST. Estimate AUD 25.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XT60 connector pair (male + female)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 pair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheaper – smallest AMASS pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress: AMASS XT60 (smallest pack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: XT60 pair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not auto-checked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power plug between the PSU and the controller – one pair is enough. Need it today? Jaycar PT4458 is ≈ $5 a pair.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small AliExpress packs ≈ US$1–2; 5 pairs ≈ US$4.96.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor axle clamp, 16 × 16 mm cross clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 16 mm cross clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part of DAZ's V2 mount – his printed parts are designed around it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical listing US$3–5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aluminium tube, 16 mm OD (cut to 100 mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kept – DAZ's exact part (shortest length)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bunnings: Metal Mate 16 mm × 1 m tube (local)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick 16 mm outside diameter and the shortest length (e.g. 250 mm); cut to 100 mm with a hacksaw. Bunnings sells a 1 m length for ≈ $6.50 if you want it today.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical 250 mm length US$2–3.50; Bunnings 16 mm × 1 m ≈ AUD 6.47 (2026 search).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quick-release clamp, Arca-Swiss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheaper – any Arca-Swiss clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress: Arca-Swiss clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How DAZ's V2 base attaches to the desk or your frame ("aluminum Quick-Release to detach from the desk"). Any Arca-Swiss clamp grips the plate below – NOT DAZ's first pick, the FANAUE lever clamp (≈ $40+). The backup is DAZ's cheaper 'option 2' listing (titled as a plate – pick its clamp option).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 search: Arca-Swiss clamps from US$6.73 (sale) ≈ AUD 10.70 incl. GST. Estimate AUD 12.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quick-release plate, Arca-Swiss, 100 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress: 100 mm Arca plate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goes with the clamp above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 search: 100 mm Arca plates from US$3.98 ≈ AUD 6.30 incl. GST.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encoder pull-up resistors, ≈1–4.7 kΩ (A, B, Z lines)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New – not on DAZ's list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress / Jaycar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress: resistors (pick 2.2K, 100 pcs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 2.2k resistors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFBeast's encoder guide says NPN encoders like the E6B2 "REQUIRES PULL UP resistors on signal lines". Value and placement per DAZ's / FFBeast's wiring diagram.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A 10–50 pack ≈ AUD 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal – steering wheel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. SHIFTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Pro Micro (ATmega32U4, 5 V / 16 MHz), USB-C</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cheaper – any seller, same size</t>
   </si>
   <si>
-    <t xml:space="preserve">AliExpress search: GT2 20T 6 mm bore</t>
+    <t xml:space="preserve">AliExpress search: Pro Micro USB-C</t>
   </si>
   <si>
     <t xml:space="preserve">Search – in-stock sellers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standard part – any seller with these sizes. Goes on the encoder shaft.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 search: GT2 20T pulleys from US$0.79 (bore varies) – about US$1 for 6 mm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GT2 closed-loop belt, 212 mm, 6 mm wide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: GT2 belt 212 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must be a closed loop, 212 mm long, 6 mm wide.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 search: 6 mm GT2 loops from US$3.04 (US store).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GT2 idler, 20T toothed, 5 mm bore, 6 mm wide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: GT2 idler 20T 5 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keeps the encoder belt tight.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ's link: US$2.24 (May 2025) ≈ AUD 3.55 incl. GST.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power supply, 24 V 10 A (240 W), AU plug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: 24V 10A power supply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The full 240 W gives the full force. Pick an enclosed 'adapter' type with an AU plug, so there's no 240 V wiring to do. Any brand works.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ's link: US$11.15 (May 2025) ≈ AUD 18 incl. GST. 2026 search: 24 V 10 A adapters with AU plug ≈ US$19 (US store) ≈ AUD 30 incl. GST. Estimate AUD 25.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XT60 connector pair (male + female)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 pair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cheaper – any seller, same size (smallest pack)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: XT60 pair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power plug between the PSU and the controller – one pair is enough. Need it today? Jaycar PT4458 is ≈ $5 a pair.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small AliExpress packs ≈ US$1–2; 5 pairs ≈ US$4.96.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor axle clamp, 16 × 16 mm cross clamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: 16 mm cross clamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Part of DAZ's V2 mount – his printed parts are designed around it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical listing US$3–5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aluminium tube, 16 mm OD (cut to 100 mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kept – DAZ's exact part (shortest length)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunnings: Metal Mate 16 mm × 1 m tube (local)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pick 16 mm outside diameter and the shortest length (e.g. 250 mm); cut to 100 mm with a hacksaw. Bunnings sells a 1 m length for ≈ $6.50 if you want it today.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical 250 mm length US$2–3.50; Bunnings 16 mm × 1 m ≈ AUD 6.47 (2026 search).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick-release clamp, Arca-Swiss (DAZ's cheaper 'option 2')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kept – DAZ's exact part (cheaper option)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: Arca-Swiss clamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How DAZ's V2 base attaches to the desk or your frame ("aluminum Quick-Release to detach from the desk"). His listing is titled as a plate – pick the clamp option; any Arca-Swiss clamp grips the plate below.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 search: Arca-Swiss clamps from US$6.73 (sale) ≈ AUD 10.70 incl. GST. Estimate AUD 12.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick-release plate, Arca-Swiss, 100 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: Arca plate 100 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goes with the clamp above.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 search: 100 mm Arca plates from US$3.98 ≈ AUD 6.30 incl. GST.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encoder pull-up resistors, ≈1–4.7 kΩ (A, B, Z lines)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New – not on DAZ's list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress / Jaycar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: 2.2k resistors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: resistor kit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFBeast's encoder guide says NPN encoders like the E6B2 "REQUIRES PULL UP resistors on signal lines". Value and placement per DAZ's / FFBeast's wiring diagram.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A 10–50 pack ≈ AUD 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal – steering wheel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. SHIFTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arduino Pro Micro (ATmega32U4, 5 V / 16 MHz), USB-C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: Pro Micro USB-C</t>
   </si>
   <si>
     <t xml:space="preserve">Must be ATmega32U4, 5 V / 16 MHz, USB-C. Runs DAZ's shifter code.</t>
@@ -2002,31 +2017,31 @@
         <f aca="false">C12*D12</f>
         <v>1.5</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="13" t="s">
         <v>42</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H12" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="I12" s="14" t="s">
-        <v>22</v>
-      </c>
       <c r="J12" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="L12" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="L12" s="9" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>47</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>19</v>
@@ -2041,31 +2056,31 @@
         <f aca="false">C13*D13</f>
         <v>3.5</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="13" t="s">
         <v>42</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H13" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="I13" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="K13" s="9" t="s">
+      <c r="L13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="L13" s="9" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>51</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>19</v>
@@ -2080,31 +2095,31 @@
         <f aca="false">C14*D14</f>
         <v>3.5</v>
       </c>
-      <c r="F14" s="16" t="s">
+      <c r="F14" s="13" t="s">
         <v>42</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H14" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I14" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J14" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="K14" s="9" t="s">
+      <c r="L14" s="9" t="s">
         <v>53</v>
-      </c>
-      <c r="L14" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>19</v>
@@ -2120,7 +2135,7 @@
         <v>25</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>21</v>
@@ -2129,24 +2144,24 @@
         <v>56</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="J15" s="15" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>1</v>
@@ -2159,30 +2174,30 @@
         <v>3</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="J16" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>19</v>
@@ -2207,24 +2222,24 @@
         <v>22</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>1</v>
@@ -2237,7 +2252,7 @@
         <v>4.5</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>21</v>
@@ -2246,21 +2261,21 @@
         <v>22</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="J18" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>19</v>
@@ -2275,31 +2290,31 @@
         <f aca="false">C19*D19</f>
         <v>12</v>
       </c>
-      <c r="F19" s="13" t="s">
-        <v>76</v>
+      <c r="F19" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>19</v>
@@ -2324,24 +2339,24 @@
         <v>22</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J20" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>1</v>
@@ -2354,30 +2369,30 @@
         <v>1</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
@@ -2396,7 +2411,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -2412,7 +2427,7 @@
     </row>
     <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>19</v>
@@ -2428,30 +2443,30 @@
         <v>7</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>19</v>
@@ -2467,30 +2482,30 @@
         <v>11</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J26" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>19</v>
@@ -2515,19 +2530,19 @@
         <v>22</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="J27" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K27" s="9"/>
       <c r="L27" s="9" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>19</v>
@@ -2552,22 +2567,22 @@
         <v>22</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="J28" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K28" s="9"/>
       <c r="L28" s="9" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>1</v>
@@ -2580,33 +2595,33 @@
         <v>4</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="I29" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J29" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="L29" s="9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="C30" s="10" t="n">
         <v>1</v>
@@ -2619,33 +2634,33 @@
         <v>4</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="I30" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J30" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="L30" s="9" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C31" s="10" t="n">
         <v>1</v>
@@ -2658,30 +2673,30 @@
         <v>4.5</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I31" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J31" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B32" s="20"/>
       <c r="C32" s="20"/>
@@ -2700,7 +2715,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -2716,7 +2731,7 @@
     </row>
     <row r="35" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B35" s="9" t="s">
         <v>19</v>
@@ -2741,21 +2756,21 @@
         <v>22</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="J35" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="L35" s="9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>19</v>
@@ -2771,30 +2786,30 @@
         <v>10</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J36" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="L36" s="9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>19</v>
@@ -2810,28 +2825,28 @@
         <v>2</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J37" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K37" s="9"/>
       <c r="L37" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>19</v>
@@ -2847,33 +2862,33 @@
         <v>5</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J38" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="L38" s="9" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>6</v>
@@ -2886,33 +2901,33 @@
         <v>8.4</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J39" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="L39" s="9" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>2</v>
@@ -2925,30 +2940,30 @@
         <v>3</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I40" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J40" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>19</v>
@@ -2973,24 +2988,24 @@
         <v>22</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="J41" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="L41" s="9" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C42" s="10" t="n">
         <v>1</v>
@@ -3012,24 +3027,24 @@
         <v>22</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="J42" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="L42" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C43" s="10" t="n">
         <v>1</v>
@@ -3042,31 +3057,31 @@
         <v>2.5</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J43" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K43" s="9"/>
       <c r="L43" s="9" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C44" s="10" t="n">
         <v>1</v>
@@ -3088,24 +3103,24 @@
         <v>22</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="J44" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L44" s="9" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C45" s="10" t="n">
         <v>1</v>
@@ -3127,19 +3142,19 @@
         <v>22</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="J45" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K45" s="9"/>
       <c r="L45" s="9" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -3158,7 +3173,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -3174,10 +3189,10 @@
     </row>
     <row r="49" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C49" s="10" t="n">
         <v>1</v>
@@ -3190,33 +3205,33 @@
         <v>1</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J49" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K49" s="9" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="L49" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C50" s="10" t="n">
         <v>1</v>
@@ -3229,31 +3244,31 @@
         <v>1</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J50" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K50" s="9"/>
       <c r="L50" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C51" s="10" t="n">
         <v>1</v>
@@ -3266,31 +3281,31 @@
         <v>1</v>
       </c>
       <c r="F51" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H51" s="14" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="I51" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J51" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K51" s="9"/>
       <c r="L51" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C52" s="10" t="n">
         <v>1</v>
@@ -3303,31 +3318,31 @@
         <v>1.5</v>
       </c>
       <c r="F52" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="I52" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J52" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K52" s="9"/>
       <c r="L52" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C53" s="10" t="n">
         <v>1</v>
@@ -3340,31 +3355,31 @@
         <v>1.5</v>
       </c>
       <c r="F53" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G53" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="I53" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J53" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K53" s="9"/>
       <c r="L53" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>1</v>
@@ -3377,31 +3392,31 @@
         <v>3</v>
       </c>
       <c r="F54" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="I54" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J54" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K54" s="9"/>
       <c r="L54" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="9" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C55" s="10" t="n">
         <v>1</v>
@@ -3414,31 +3429,31 @@
         <v>1.5</v>
       </c>
       <c r="F55" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J55" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K55" s="9"/>
       <c r="L55" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C56" s="10" t="n">
         <v>1</v>
@@ -3451,31 +3466,31 @@
         <v>1.5</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H56" s="14" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="I56" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J56" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K56" s="9"/>
       <c r="L56" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="B57" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="B57" s="9" t="s">
-        <v>194</v>
       </c>
       <c r="C57" s="10" t="n">
         <v>1</v>
@@ -3488,31 +3503,31 @@
         <v>1</v>
       </c>
       <c r="F57" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="14" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="I57" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J57" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K57" s="9"/>
       <c r="L57" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C58" s="10" t="n">
         <v>1</v>
@@ -3525,31 +3540,31 @@
         <v>1.5</v>
       </c>
       <c r="F58" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="I58" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J58" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K58" s="9"/>
       <c r="L58" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="C59" s="10" t="n">
         <v>1</v>
@@ -3562,31 +3577,31 @@
         <v>1.5</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G59" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H59" s="14" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="I59" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J59" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K59" s="9"/>
       <c r="L59" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C60" s="10" t="n">
         <v>1</v>
@@ -3599,31 +3614,31 @@
         <v>2.5</v>
       </c>
       <c r="F60" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G60" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H60" s="14" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I60" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J60" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K60" s="9"/>
       <c r="L60" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C61" s="10" t="n">
         <v>1</v>
@@ -3636,31 +3651,31 @@
         <v>2</v>
       </c>
       <c r="F61" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G61" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H61" s="14" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="I61" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J61" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K61" s="9"/>
       <c r="L61" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C62" s="10" t="n">
         <v>1</v>
@@ -3673,31 +3688,31 @@
         <v>2</v>
       </c>
       <c r="F62" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G62" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H62" s="14" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="I62" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J62" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K62" s="9"/>
       <c r="L62" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C63" s="10" t="n">
         <v>1</v>
@@ -3710,31 +3725,31 @@
         <v>2</v>
       </c>
       <c r="F63" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G63" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H63" s="14" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="I63" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J63" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K63" s="9"/>
       <c r="L63" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C64" s="10" t="n">
         <v>1</v>
@@ -3747,31 +3762,31 @@
         <v>2</v>
       </c>
       <c r="F64" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G64" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H64" s="14" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="I64" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J64" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K64" s="9"/>
       <c r="L64" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C65" s="10" t="n">
         <v>1</v>
@@ -3784,31 +3799,31 @@
         <v>1</v>
       </c>
       <c r="F65" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G65" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H65" s="14" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="I65" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J65" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K65" s="9"/>
       <c r="L65" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C66" s="10" t="n">
         <v>1</v>
@@ -3821,31 +3836,31 @@
         <v>1.5</v>
       </c>
       <c r="F66" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G66" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H66" s="14" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="I66" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J66" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K66" s="9"/>
       <c r="L66" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C67" s="10" t="n">
         <v>1</v>
@@ -3858,31 +3873,31 @@
         <v>1</v>
       </c>
       <c r="F67" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G67" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H67" s="14" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="I67" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J67" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K67" s="9"/>
       <c r="L67" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C68" s="10" t="n">
         <v>1</v>
@@ -3895,31 +3910,31 @@
         <v>1</v>
       </c>
       <c r="F68" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G68" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H68" s="14" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="I68" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J68" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K68" s="9"/>
       <c r="L68" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C69" s="10" t="n">
         <v>1</v>
@@ -3932,29 +3947,29 @@
         <v>1.5</v>
       </c>
       <c r="F69" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G69" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H69" s="14" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="I69" s="17"/>
       <c r="J69" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K69" s="9"/>
       <c r="L69" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C70" s="10" t="n">
         <v>1</v>
@@ -3967,29 +3982,29 @@
         <v>1</v>
       </c>
       <c r="F70" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G70" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H70" s="14" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I70" s="17"/>
       <c r="J70" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K70" s="9"/>
       <c r="L70" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="9" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C71" s="10" t="n">
         <v>7</v>
@@ -4002,33 +4017,33 @@
         <v>7</v>
       </c>
       <c r="F71" s="16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G71" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H71" s="14" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="I71" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J71" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K71" s="9" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="L71" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="9" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C72" s="10" t="n">
         <v>1</v>
@@ -4041,31 +4056,31 @@
         <v>2.5</v>
       </c>
       <c r="F72" s="13" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="H72" s="14" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="I72" s="17"/>
       <c r="J72" s="15" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="K72" s="9" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="L72" s="9" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="9" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C73" s="10" t="n">
         <v>1</v>
@@ -4078,30 +4093,30 @@
         <v>3.5</v>
       </c>
       <c r="F73" s="16" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="H73" s="14" t="s">
         <v>22</v>
       </c>
       <c r="I73" s="14" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="J73" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K73" s="9" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="L73" s="9" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="19" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B74" s="20"/>
       <c r="C74" s="20"/>
@@ -4120,7 +4135,7 @@
     </row>
     <row r="76" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="22" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B76" s="22"/>
       <c r="C76" s="22"/>
@@ -4139,7 +4154,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B78" s="8"/>
       <c r="C78" s="8"/>
@@ -4155,10 +4170,10 @@
     </row>
     <row r="79" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="9" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C79" s="10" t="n">
         <v>1</v>
@@ -4171,33 +4186,33 @@
         <v>6</v>
       </c>
       <c r="F79" s="16" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="H79" s="14" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="I79" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J79" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K79" s="9" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="L79" s="9" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="9" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C80" s="10" t="n">
         <v>1</v>
@@ -4210,30 +4225,30 @@
         <v>4</v>
       </c>
       <c r="F80" s="16" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="H80" s="14" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="I80" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J80" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K80" s="9" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="L80" s="9" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="9" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="B81" s="9" t="s">
         <v>19</v>
@@ -4249,31 +4264,31 @@
         <v>12</v>
       </c>
       <c r="F81" s="16" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="H81" s="14" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="I81" s="17"/>
       <c r="J81" s="15" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="K81" s="9" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="L81" s="9" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="9" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C82" s="10" t="n">
         <v>1</v>
@@ -4286,27 +4301,27 @@
         <v>5</v>
       </c>
       <c r="F82" s="24" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="H82" s="17"/>
       <c r="I82" s="17"/>
       <c r="J82" s="15"/>
       <c r="K82" s="9" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="L82" s="9" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="9" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C83" s="10" t="n">
         <v>3</v>
@@ -4319,24 +4334,24 @@
         <v>6</v>
       </c>
       <c r="F83" s="24" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="H83" s="17"/>
       <c r="I83" s="17"/>
       <c r="J83" s="15"/>
       <c r="K83" s="9" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="L83" s="9" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="19" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="B84" s="20"/>
       <c r="C84" s="20"/>
@@ -4355,7 +4370,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="E85" s="6" t="n">
         <f aca="false">E76+E84</f>
@@ -4364,7 +4379,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="8" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B87" s="8"/>
       <c r="C87" s="8"/>
@@ -4380,7 +4395,7 @@
     </row>
     <row r="88" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="9" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="B88" s="9" t="s">
         <v>19</v>
@@ -4396,7 +4411,7 @@
         <v>10</v>
       </c>
       <c r="F88" s="25" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="G88" s="9" t="s">
         <v>21</v>
@@ -4405,24 +4420,24 @@
         <v>22</v>
       </c>
       <c r="I88" s="14" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="J88" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K88" s="9" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="L88" s="9" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="9" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C89" s="10" t="n">
         <v>2</v>
@@ -4435,7 +4450,7 @@
         <v>6</v>
       </c>
       <c r="F89" s="25" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="G89" s="9" t="s">
         <v>21</v>
@@ -4444,24 +4459,24 @@
         <v>22</v>
       </c>
       <c r="I89" s="14" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="J89" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K89" s="9" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="L89" s="9" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="9" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="B90" s="9" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="C90" s="10" t="n">
         <v>1</v>
@@ -4474,7 +4489,7 @@
         <v>5</v>
       </c>
       <c r="F90" s="25" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="G90" s="9" t="s">
         <v>21</v>
@@ -4483,21 +4498,21 @@
         <v>22</v>
       </c>
       <c r="I90" s="14" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="J90" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K90" s="9" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="L90" s="9" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="9" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B91" s="9" t="s">
         <v>19</v>
@@ -4513,7 +4528,7 @@
         <v>1.5</v>
       </c>
       <c r="F91" s="25" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="G91" s="9" t="s">
         <v>21</v>
@@ -4522,24 +4537,24 @@
         <v>22</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="J91" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K91" s="9" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="L91" s="9" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="9" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C92" s="10" t="n">
         <v>1</v>
@@ -4552,33 +4567,33 @@
         <v>0</v>
       </c>
       <c r="F92" s="25" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="H92" s="14" t="s">
         <v>22</v>
       </c>
       <c r="I92" s="14" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="J92" s="15" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="K92" s="9" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="L92" s="9" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="9" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B93" s="9" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C93" s="10" t="n">
         <v>1</v>
@@ -4591,24 +4606,24 @@
         <v>2</v>
       </c>
       <c r="F93" s="25" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="G93" s="9" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="H93" s="17"/>
       <c r="I93" s="17"/>
       <c r="J93" s="15"/>
       <c r="K93" s="9" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="L93" s="9" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="19" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B94" s="20"/>
       <c r="C94" s="20"/>
@@ -4627,7 +4642,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="E95" s="6" t="n">
         <f aca="false">E76+E94</f>
@@ -4636,7 +4651,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="8" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
@@ -4652,10 +4667,10 @@
     </row>
     <row r="98" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="9" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C98" s="10" t="n">
         <v>1</v>
@@ -4668,27 +4683,27 @@
         <v>18</v>
       </c>
       <c r="F98" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="H98" s="17"/>
       <c r="I98" s="17"/>
       <c r="J98" s="15"/>
       <c r="K98" s="9" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="L98" s="9" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="9" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C99" s="10" t="n">
         <v>1</v>
@@ -4701,27 +4716,27 @@
         <v>25</v>
       </c>
       <c r="F99" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G99" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="H99" s="17"/>
       <c r="I99" s="17"/>
       <c r="J99" s="15"/>
       <c r="K99" s="9" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="L99" s="9" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B100" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C100" s="10" t="n">
         <v>1</v>
@@ -4734,27 +4749,27 @@
         <v>7</v>
       </c>
       <c r="F100" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="H100" s="17"/>
       <c r="I100" s="17"/>
       <c r="J100" s="15"/>
       <c r="K100" s="9" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="L100" s="9" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="9" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C101" s="10" t="n">
         <v>1</v>
@@ -4767,31 +4782,31 @@
         <v>38</v>
       </c>
       <c r="F101" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G101" s="9" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H101" s="14" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="I101" s="17"/>
       <c r="J101" s="15" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="K101" s="9" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="L101" s="9" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="9" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B102" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C102" s="10" t="n">
         <v>1</v>
@@ -4804,31 +4819,31 @@
         <v>15</v>
       </c>
       <c r="F102" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G102" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H102" s="14" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="I102" s="17"/>
       <c r="J102" s="15" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="K102" s="9" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="L102" s="9" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="9" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B103" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C103" s="10" t="n">
         <v>1</v>
@@ -4841,27 +4856,27 @@
         <v>25</v>
       </c>
       <c r="F103" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G103" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="H103" s="17"/>
       <c r="I103" s="17"/>
       <c r="J103" s="15"/>
       <c r="K103" s="9" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="L103" s="9" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="9" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B104" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C104" s="10" t="n">
         <v>1</v>
@@ -4874,24 +4889,24 @@
         <v>4.3</v>
       </c>
       <c r="F104" s="26" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="H104" s="17"/>
       <c r="I104" s="17"/>
       <c r="J104" s="15"/>
       <c r="K104" s="9" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="L104" s="9" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="19" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B105" s="20"/>
       <c r="C105" s="20"/>
@@ -4910,7 +4925,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="E106" s="6" t="n">
         <f aca="false">E76-E105</f>
@@ -4919,7 +4934,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="8" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B108" s="8"/>
       <c r="C108" s="8"/>
@@ -4935,7 +4950,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="27" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B109" s="27"/>
       <c r="C109" s="27"/>
@@ -4951,7 +4966,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="27" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="B110" s="27"/>
       <c r="C110" s="27"/>
@@ -4967,7 +4982,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="27" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B111" s="27"/>
       <c r="C111" s="27"/>
@@ -4983,7 +4998,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="8" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B113" s="8"/>
       <c r="C113" s="8"/>
@@ -4999,7 +5014,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="28" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="B114" s="28"/>
       <c r="C114" s="28"/>
@@ -5015,7 +5030,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="28" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B115" s="28"/>
       <c r="C115" s="28"/>
@@ -5031,7 +5046,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="28" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B116" s="28"/>
       <c r="C116" s="28"/>
@@ -5047,7 +5062,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="28" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="B117" s="28"/>
       <c r="C117" s="28"/>
@@ -5063,7 +5078,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="28" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B118" s="28"/>
       <c r="C118" s="28"/>
@@ -5079,7 +5094,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="28" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B119" s="28"/>
       <c r="C119" s="28"/>
@@ -5128,26 +5143,26 @@
     <hyperlink ref="I10" r:id="rId4" display="AliExpress search: E6B2-CWZ6C"/>
     <hyperlink ref="H11" r:id="rId5" display="AliExpress – DAZ's link"/>
     <hyperlink ref="I11" r:id="rId6" display="AliExpress search: 13&quot; flat wheel"/>
-    <hyperlink ref="H12" r:id="rId7" display="AliExpress search: GT2 20T 6 mm bore"/>
-    <hyperlink ref="I12" r:id="rId8" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H13" r:id="rId9" display="AliExpress search: GT2 belt 212 mm"/>
-    <hyperlink ref="I13" r:id="rId10" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H14" r:id="rId11" display="AliExpress search: GT2 idler 20T 5 mm"/>
-    <hyperlink ref="I14" r:id="rId12" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H15" r:id="rId13" display="AliExpress search: 24V 10A power supply"/>
-    <hyperlink ref="I15" r:id="rId14" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H16" r:id="rId15" display="AliExpress search: XT60 pair"/>
-    <hyperlink ref="I16" r:id="rId16" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H12" r:id="rId7" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I12" r:id="rId8" display="AliExpress search: GT2 20T 6 mm bore"/>
+    <hyperlink ref="H13" r:id="rId9" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I13" r:id="rId10" display="AliExpress search: GT2 belt 212 mm"/>
+    <hyperlink ref="H14" r:id="rId11" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I14" r:id="rId12" display="AliExpress search: GT2 idler 20T 5 mm"/>
+    <hyperlink ref="H15" r:id="rId13" display="AliExpress: 24 V adapter (pick 10A, AU plug)"/>
+    <hyperlink ref="I15" r:id="rId14" display="AliExpress search: 24V 10A power supply"/>
+    <hyperlink ref="H16" r:id="rId15" display="AliExpress: AMASS XT60 (smallest pack)"/>
+    <hyperlink ref="I16" r:id="rId16" display="AliExpress search: XT60 pair"/>
     <hyperlink ref="H17" r:id="rId17" display="AliExpress – DAZ's link"/>
     <hyperlink ref="I17" r:id="rId18" display="AliExpress search: 16 mm cross clamp"/>
     <hyperlink ref="H18" r:id="rId19" display="AliExpress – DAZ's link"/>
     <hyperlink ref="I18" r:id="rId20" display="Bunnings: Metal Mate 16 mm × 1 m tube (local)"/>
-    <hyperlink ref="H19" r:id="rId21" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="I19" r:id="rId22" display="AliExpress search: Arca-Swiss clamp"/>
+    <hyperlink ref="H19" r:id="rId21" display="AliExpress: Arca-Swiss clamp"/>
+    <hyperlink ref="I19" r:id="rId22" display="AliExpress – DAZ's link"/>
     <hyperlink ref="H20" r:id="rId23" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="I20" r:id="rId24" display="AliExpress search: Arca plate 100 mm"/>
-    <hyperlink ref="H21" r:id="rId25" display="AliExpress search: 2.2k resistors"/>
-    <hyperlink ref="I21" r:id="rId26" display="AliExpress search: resistor kit"/>
+    <hyperlink ref="I20" r:id="rId24" display="AliExpress: 100 mm Arca plate"/>
+    <hyperlink ref="H21" r:id="rId25" display="AliExpress: resistors (pick 2.2K, 100 pcs)"/>
+    <hyperlink ref="I21" r:id="rId26" display="AliExpress search: 2.2k resistors"/>
     <hyperlink ref="H25" r:id="rId27" display="AliExpress search: Pro Micro USB-C"/>
     <hyperlink ref="I25" r:id="rId28" display="AliExpress – DAZ's link"/>
     <hyperlink ref="H26" r:id="rId29" display="AliExpress search: MGN12H 100 mm"/>

</xml_diff>

<commit_message>
Confirm every wheel cart listing is live; fix XT60 and self-tapper options
- All 23 AliExpress listings in the wheel cart list were opened on 3 Oct
  2026 and confirmed live (resistor pack, XT60H pack, Arca-Swiss clamp
  and plate, DAZ's screw and nut listings, etc.).
- The XT60 listing only sells 5-pair packs, so its target is now AUD 5
  (or one pair from Jaycar). The wheel is about AUD 193 and all three
  about AUD 330.
- Self-tapping options now use the ST sizes the listing actually sells.
- Formatting fixes for the shipping row and the "don't add" block.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEYLvGWigrKvVwvVek2yBU
</commit_message>
<xml_diff>
--- a/parts-lists/DAZ_all_three_best_value_parts_list_AUD.xlsx
+++ b/parts-lists/DAZ_all_three_best_value_parts_list_AUD.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="364">
   <si>
     <t xml:space="preserve">DAZ wheel + shifter + pedals – best-value parts list for all three (AUD)</t>
   </si>
@@ -211,22 +211,19 @@
     <t xml:space="preserve">1 pair</t>
   </si>
   <si>
-    <t xml:space="preserve">Cheaper – smallest AMASS pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress: AMASS XT60 (smallest pack)</t>
+    <t xml:space="preserve">Cheaper – smallest pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress: XT60H (10 pcs = 5 pairs)</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress search: XT60 pair</t>
   </si>
   <si>
-    <t xml:space="preserve">Not auto-checked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power plug between the PSU and the controller – one pair is enough. Need it today? Jaycar PT4458 is ≈ $5 a pair.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small AliExpress packs ≈ US$1–2; 5 pairs ≈ US$4.96.</t>
+    <t xml:space="preserve">Power plug between the PSU and the controller – you need one pair; this listing's smallest pack is 5 pairs. Or get a single pair from Jaycar (PT4458, ≈ $5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 search: XT60H 5-pair packs ≈ US$4.96 (US store).</t>
   </si>
   <si>
     <t xml:space="preserve">Motor axle clamp, 16 × 16 mm cross clamp</t>
@@ -1773,11 +1770,11 @@
       </c>
       <c r="E3" s="6" t="n">
         <f aca="false">E76</f>
-        <v>328.4</v>
+        <v>330.4</v>
       </c>
       <c r="F3" s="3" t="str">
         <f aca="false">IF($E$3&lt;=$B$3,"UNDER BUDGET – $"&amp;TEXT($B$3-$E$3,"0.00")&amp;" spare","OVER BUDGET by $"&amp;TEXT($E$3-$B$3,"0.00"))</f>
-        <v>OVER BUDGET by $228.40</v>
+        <v>OVER BUDGET by $230.40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1789,11 +1786,11 @@
       </c>
       <c r="E4" s="6" t="n">
         <f aca="false">E106</f>
-        <v>196.1</v>
+        <v>198.1</v>
       </c>
       <c r="F4" s="3" t="str">
         <f aca="false">IF($E$4&lt;=$B$3,"UNDER BUDGET – $"&amp;TEXT($B$3-$E$4,"0.00")&amp;" spare","OVER BUDGET by $"&amp;TEXT($E$4-$B$3,"0.00"))</f>
-        <v>OVER BUDGET by $96.10</v>
+        <v>OVER BUDGET by $98.10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2156,7 +2153,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>60</v>
       </c>
@@ -2167,11 +2164,11 @@
         <v>1</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">C16*D16</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>62</v>
@@ -2186,18 +2183,18 @@
         <v>64</v>
       </c>
       <c r="J16" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K16" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="9" t="s">
+      <c r="L16" s="9" t="s">
         <v>66</v>
-      </c>
-      <c r="L16" s="9" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>19</v>
@@ -2222,24 +2219,24 @@
         <v>22</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K17" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="L17" s="9" t="s">
         <v>70</v>
-      </c>
-      <c r="L17" s="9" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>73</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>1</v>
@@ -2252,30 +2249,30 @@
         <v>4.5</v>
       </c>
       <c r="F18" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="14" t="s">
         <v>74</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>75</v>
       </c>
       <c r="J18" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K18" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="L18" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="L18" s="9" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>19</v>
@@ -2291,30 +2288,30 @@
         <v>12</v>
       </c>
       <c r="F19" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="G19" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="14" t="s">
+      <c r="I19" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="I19" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="K19" s="9" t="s">
+      <c r="L19" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="L19" s="9" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>19</v>
@@ -2339,24 +2336,24 @@
         <v>22</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J20" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K20" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L20" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="L20" s="9" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>87</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>88</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>1</v>
@@ -2369,37 +2366,37 @@
         <v>1</v>
       </c>
       <c r="F21" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="G21" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="H21" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="I21" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="I21" s="14" t="s">
+      <c r="J21" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K21" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="J21" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="K21" s="9" t="s">
+      <c r="L21" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="L21" s="9" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
       <c r="E22" s="21" t="n">
         <f aca="false">SUM(E8:E21)</f>
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F22" s="20"/>
       <c r="G22" s="20"/>
@@ -2411,7 +2408,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -2427,7 +2424,7 @@
     </row>
     <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>19</v>
@@ -2443,30 +2440,30 @@
         <v>7</v>
       </c>
       <c r="F25" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="G25" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H25" s="14" t="s">
+      <c r="I25" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J25" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="I25" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="15" t="s">
+      <c r="K25" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="K25" s="9" t="s">
+      <c r="L25" s="9" t="s">
         <v>101</v>
-      </c>
-      <c r="L25" s="9" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>19</v>
@@ -2482,30 +2479,30 @@
         <v>11</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H26" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K26" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="I26" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K26" s="9" t="s">
+      <c r="L26" s="9" t="s">
         <v>105</v>
-      </c>
-      <c r="L26" s="9" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>19</v>
@@ -2530,19 +2527,19 @@
         <v>22</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J27" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K27" s="9"/>
       <c r="L27" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>19</v>
@@ -2567,22 +2564,22 @@
         <v>22</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J28" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K28" s="9"/>
       <c r="L28" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>112</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>113</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>1</v>
@@ -2595,33 +2592,33 @@
         <v>4</v>
       </c>
       <c r="F29" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H29" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K29" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="I29" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K29" s="9" t="s">
+      <c r="L29" s="9" t="s">
         <v>115</v>
-      </c>
-      <c r="L29" s="9" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>117</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>118</v>
       </c>
       <c r="C30" s="10" t="n">
         <v>1</v>
@@ -2634,33 +2631,33 @@
         <v>4</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H30" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J30" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K30" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="I30" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J30" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K30" s="9" t="s">
+      <c r="L30" s="9" t="s">
         <v>120</v>
-      </c>
-      <c r="L30" s="9" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" s="9" t="s">
         <v>122</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>123</v>
       </c>
       <c r="C31" s="10" t="n">
         <v>1</v>
@@ -2673,30 +2670,30 @@
         <v>4.5</v>
       </c>
       <c r="F31" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H31" s="14" t="s">
+      <c r="I31" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J31" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K31" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="I31" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J31" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K31" s="9" t="s">
+      <c r="L31" s="9" t="s">
         <v>126</v>
-      </c>
-      <c r="L31" s="9" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B32" s="20"/>
       <c r="C32" s="20"/>
@@ -2715,7 +2712,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -2731,7 +2728,7 @@
     </row>
     <row r="35" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B35" s="9" t="s">
         <v>19</v>
@@ -2756,21 +2753,21 @@
         <v>22</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J35" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K35" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="L35" s="9" t="s">
         <v>132</v>
-      </c>
-      <c r="L35" s="9" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>19</v>
@@ -2786,30 +2783,30 @@
         <v>10</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H36" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J36" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K36" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="I36" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J36" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K36" s="9" t="s">
+      <c r="L36" s="9" t="s">
         <v>136</v>
-      </c>
-      <c r="L36" s="9" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>19</v>
@@ -2825,28 +2822,28 @@
         <v>2</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J37" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K37" s="9"/>
       <c r="L37" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>19</v>
@@ -2862,33 +2859,33 @@
         <v>5</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H38" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K38" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="I38" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J38" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K38" s="9" t="s">
+      <c r="L38" s="9" t="s">
         <v>143</v>
-      </c>
-      <c r="L38" s="9" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B39" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>6</v>
@@ -2901,33 +2898,33 @@
         <v>8.4</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H39" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="I39" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J39" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K39" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="I39" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J39" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K39" s="9" t="s">
+      <c r="L39" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="L39" s="9" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B40" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>151</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>2</v>
@@ -2940,30 +2937,30 @@
         <v>3</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H40" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K40" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="I40" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J40" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K40" s="9" t="s">
+      <c r="L40" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="L40" s="9" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>19</v>
@@ -2988,24 +2985,24 @@
         <v>22</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J41" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K41" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="L41" s="9" t="s">
         <v>157</v>
-      </c>
-      <c r="L41" s="9" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>159</v>
-      </c>
-      <c r="B42" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="C42" s="10" t="n">
         <v>1</v>
@@ -3027,24 +3024,24 @@
         <v>22</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J42" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K42" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="L42" s="9" t="s">
         <v>162</v>
-      </c>
-      <c r="L42" s="9" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B43" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="C43" s="10" t="n">
         <v>1</v>
@@ -3057,31 +3054,31 @@
         <v>2.5</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J43" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K43" s="9"/>
       <c r="L43" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="B44" s="9" t="s">
         <v>168</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>169</v>
       </c>
       <c r="C44" s="10" t="n">
         <v>1</v>
@@ -3103,24 +3100,24 @@
         <v>22</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J44" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K44" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="L44" s="9" t="s">
         <v>171</v>
-      </c>
-      <c r="L44" s="9" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C45" s="10" t="n">
         <v>1</v>
@@ -3142,19 +3139,19 @@
         <v>22</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J45" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K45" s="9"/>
       <c r="L45" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -3173,7 +3170,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -3189,10 +3186,10 @@
     </row>
     <row r="49" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B49" s="9" t="s">
         <v>178</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>179</v>
       </c>
       <c r="C49" s="10" t="n">
         <v>1</v>
@@ -3205,33 +3202,33 @@
         <v>1</v>
       </c>
       <c r="F49" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H49" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="G49" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H49" s="14" t="s">
+      <c r="I49" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J49" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K49" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="I49" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J49" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K49" s="9" t="s">
+      <c r="L49" s="9" t="s">
         <v>182</v>
-      </c>
-      <c r="L49" s="9" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="B50" s="9" t="s">
         <v>184</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>185</v>
       </c>
       <c r="C50" s="10" t="n">
         <v>1</v>
@@ -3244,31 +3241,31 @@
         <v>1</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J50" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K50" s="9"/>
       <c r="L50" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B51" s="9" t="s">
         <v>187</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>188</v>
       </c>
       <c r="C51" s="10" t="n">
         <v>1</v>
@@ -3281,31 +3278,31 @@
         <v>1</v>
       </c>
       <c r="F51" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H51" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="I51" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J51" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K51" s="9"/>
       <c r="L51" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C52" s="10" t="n">
         <v>1</v>
@@ -3318,31 +3315,31 @@
         <v>1.5</v>
       </c>
       <c r="F52" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I52" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J52" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K52" s="9"/>
       <c r="L52" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="B53" s="9" t="s">
         <v>192</v>
-      </c>
-      <c r="B53" s="9" t="s">
-        <v>193</v>
       </c>
       <c r="C53" s="10" t="n">
         <v>1</v>
@@ -3355,31 +3352,31 @@
         <v>1.5</v>
       </c>
       <c r="F53" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G53" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I53" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J53" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K53" s="9"/>
       <c r="L53" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B54" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="B54" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>1</v>
@@ -3392,31 +3389,31 @@
         <v>3</v>
       </c>
       <c r="F54" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I54" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J54" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K54" s="9"/>
       <c r="L54" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B55" s="9" t="s">
         <v>198</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>199</v>
       </c>
       <c r="C55" s="10" t="n">
         <v>1</v>
@@ -3429,31 +3426,31 @@
         <v>1.5</v>
       </c>
       <c r="F55" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J55" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K55" s="9"/>
       <c r="L55" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="B56" s="9" t="s">
         <v>201</v>
-      </c>
-      <c r="B56" s="9" t="s">
-        <v>202</v>
       </c>
       <c r="C56" s="10" t="n">
         <v>1</v>
@@ -3466,31 +3463,31 @@
         <v>1.5</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H56" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I56" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J56" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K56" s="9"/>
       <c r="L56" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C57" s="10" t="n">
         <v>1</v>
@@ -3503,31 +3500,31 @@
         <v>1</v>
       </c>
       <c r="F57" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I57" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J57" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K57" s="9"/>
       <c r="L57" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B58" s="9" t="s">
         <v>206</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>207</v>
       </c>
       <c r="C58" s="10" t="n">
         <v>1</v>
@@ -3540,31 +3537,31 @@
         <v>1.5</v>
       </c>
       <c r="F58" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I58" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J58" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K58" s="9"/>
       <c r="L58" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B59" s="9" t="s">
         <v>209</v>
-      </c>
-      <c r="B59" s="9" t="s">
-        <v>210</v>
       </c>
       <c r="C59" s="10" t="n">
         <v>1</v>
@@ -3577,31 +3574,31 @@
         <v>1.5</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G59" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H59" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I59" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J59" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K59" s="9"/>
       <c r="L59" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B60" s="9" t="s">
         <v>212</v>
-      </c>
-      <c r="B60" s="9" t="s">
-        <v>213</v>
       </c>
       <c r="C60" s="10" t="n">
         <v>1</v>
@@ -3614,31 +3611,31 @@
         <v>2.5</v>
       </c>
       <c r="F60" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G60" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H60" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I60" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J60" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K60" s="9"/>
       <c r="L60" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C61" s="10" t="n">
         <v>1</v>
@@ -3651,31 +3648,31 @@
         <v>2</v>
       </c>
       <c r="F61" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G61" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H61" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I61" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J61" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K61" s="9"/>
       <c r="L61" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C62" s="10" t="n">
         <v>1</v>
@@ -3688,31 +3685,31 @@
         <v>2</v>
       </c>
       <c r="F62" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G62" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H62" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I62" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J62" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K62" s="9"/>
       <c r="L62" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="B63" s="9" t="s">
         <v>219</v>
-      </c>
-      <c r="B63" s="9" t="s">
-        <v>220</v>
       </c>
       <c r="C63" s="10" t="n">
         <v>1</v>
@@ -3725,31 +3722,31 @@
         <v>2</v>
       </c>
       <c r="F63" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G63" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H63" s="14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I63" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J63" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K63" s="9"/>
       <c r="L63" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C64" s="10" t="n">
         <v>1</v>
@@ -3762,31 +3759,31 @@
         <v>2</v>
       </c>
       <c r="F64" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G64" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H64" s="14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I64" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J64" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K64" s="9"/>
       <c r="L64" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C65" s="10" t="n">
         <v>1</v>
@@ -3799,31 +3796,31 @@
         <v>1</v>
       </c>
       <c r="F65" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G65" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H65" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I65" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J65" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K65" s="9"/>
       <c r="L65" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B66" s="9" t="s">
         <v>226</v>
-      </c>
-      <c r="B66" s="9" t="s">
-        <v>227</v>
       </c>
       <c r="C66" s="10" t="n">
         <v>1</v>
@@ -3836,31 +3833,31 @@
         <v>1.5</v>
       </c>
       <c r="F66" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G66" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H66" s="14" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I66" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J66" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K66" s="9"/>
       <c r="L66" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="B67" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="C67" s="10" t="n">
         <v>1</v>
@@ -3873,31 +3870,31 @@
         <v>1</v>
       </c>
       <c r="F67" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G67" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H67" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I67" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J67" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K67" s="9"/>
       <c r="L67" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>232</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>233</v>
       </c>
       <c r="C68" s="10" t="n">
         <v>1</v>
@@ -3910,31 +3907,31 @@
         <v>1</v>
       </c>
       <c r="F68" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G68" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H68" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I68" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J68" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K68" s="9"/>
       <c r="L68" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B69" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="B69" s="9" t="s">
-        <v>236</v>
       </c>
       <c r="C69" s="10" t="n">
         <v>1</v>
@@ -3947,29 +3944,29 @@
         <v>1.5</v>
       </c>
       <c r="F69" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G69" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H69" s="14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I69" s="17"/>
       <c r="J69" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K69" s="9"/>
       <c r="L69" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="B70" s="9" t="s">
         <v>238</v>
-      </c>
-      <c r="B70" s="9" t="s">
-        <v>239</v>
       </c>
       <c r="C70" s="10" t="n">
         <v>1</v>
@@ -3982,29 +3979,29 @@
         <v>1</v>
       </c>
       <c r="F70" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G70" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H70" s="14" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I70" s="17"/>
       <c r="J70" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K70" s="9"/>
       <c r="L70" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B71" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>242</v>
       </c>
       <c r="C71" s="10" t="n">
         <v>7</v>
@@ -4017,33 +4014,33 @@
         <v>7</v>
       </c>
       <c r="F71" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G71" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H71" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="I71" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J71" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K71" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="I71" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J71" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K71" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="L71" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B72" s="9" t="s">
         <v>245</v>
-      </c>
-      <c r="B72" s="9" t="s">
-        <v>246</v>
       </c>
       <c r="C72" s="10" t="n">
         <v>1</v>
@@ -4056,31 +4053,31 @@
         <v>2.5</v>
       </c>
       <c r="F72" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="G72" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="G72" s="9" t="s">
+      <c r="H72" s="14" t="s">
         <v>248</v>
-      </c>
-      <c r="H72" s="14" t="s">
-        <v>249</v>
       </c>
       <c r="I72" s="17"/>
       <c r="J72" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="K72" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="K72" s="9" t="s">
+      <c r="L72" s="9" t="s">
         <v>251</v>
-      </c>
-      <c r="L72" s="9" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="B73" s="9" t="s">
         <v>253</v>
-      </c>
-      <c r="B73" s="9" t="s">
-        <v>254</v>
       </c>
       <c r="C73" s="10" t="n">
         <v>1</v>
@@ -4093,30 +4090,30 @@
         <v>3.5</v>
       </c>
       <c r="F73" s="16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G73" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="H73" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I73" s="14" t="s">
         <v>255</v>
-      </c>
-      <c r="H73" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="I73" s="14" t="s">
-        <v>256</v>
       </c>
       <c r="J73" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K73" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="L73" s="9" t="s">
         <v>257</v>
-      </c>
-      <c r="L73" s="9" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B74" s="20"/>
       <c r="C74" s="20"/>
@@ -4135,14 +4132,14 @@
     </row>
     <row r="76" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="22" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B76" s="22"/>
       <c r="C76" s="22"/>
       <c r="D76" s="22"/>
       <c r="E76" s="23" t="n">
         <f aca="false">E22+E32+E46+E74</f>
-        <v>328.4</v>
+        <v>330.4</v>
       </c>
       <c r="F76" s="22"/>
       <c r="G76" s="22"/>
@@ -4154,7 +4151,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B78" s="8"/>
       <c r="C78" s="8"/>
@@ -4170,10 +4167,10 @@
     </row>
     <row r="79" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C79" s="10" t="n">
         <v>1</v>
@@ -4186,33 +4183,33 @@
         <v>6</v>
       </c>
       <c r="F79" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="G79" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="G79" s="9" t="s">
+      <c r="H79" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="H79" s="14" t="s">
+      <c r="I79" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J79" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K79" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="I79" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J79" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K79" s="9" t="s">
+      <c r="L79" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="L79" s="9" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C80" s="10" t="n">
         <v>1</v>
@@ -4225,30 +4222,30 @@
         <v>4</v>
       </c>
       <c r="F80" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="G80" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="G80" s="9" t="s">
+      <c r="H80" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="H80" s="14" t="s">
+      <c r="I80" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J80" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="K80" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="I80" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J80" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K80" s="9" t="s">
+      <c r="L80" s="9" t="s">
         <v>272</v>
-      </c>
-      <c r="L80" s="9" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B81" s="9" t="s">
         <v>19</v>
@@ -4264,31 +4261,31 @@
         <v>12</v>
       </c>
       <c r="F81" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="G81" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="G81" s="9" t="s">
+      <c r="H81" s="14" t="s">
         <v>276</v>
-      </c>
-      <c r="H81" s="14" t="s">
-        <v>277</v>
       </c>
       <c r="I81" s="17"/>
       <c r="J81" s="15" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K81" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="L81" s="9" t="s">
         <v>278</v>
-      </c>
-      <c r="L81" s="9" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="B82" s="9" t="s">
         <v>280</v>
-      </c>
-      <c r="B82" s="9" t="s">
-        <v>281</v>
       </c>
       <c r="C82" s="10" t="n">
         <v>1</v>
@@ -4301,27 +4298,27 @@
         <v>5</v>
       </c>
       <c r="F82" s="24" t="s">
+        <v>281</v>
+      </c>
+      <c r="G82" s="9" t="s">
         <v>282</v>
-      </c>
-      <c r="G82" s="9" t="s">
-        <v>283</v>
       </c>
       <c r="H82" s="17"/>
       <c r="I82" s="17"/>
       <c r="J82" s="15"/>
       <c r="K82" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="L82" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="L82" s="9" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C83" s="10" t="n">
         <v>3</v>
@@ -4334,24 +4331,24 @@
         <v>6</v>
       </c>
       <c r="F83" s="24" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H83" s="17"/>
       <c r="I83" s="17"/>
       <c r="J83" s="15"/>
       <c r="K83" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="L83" s="9" t="s">
         <v>288</v>
-      </c>
-      <c r="L83" s="9" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B84" s="20"/>
       <c r="C84" s="20"/>
@@ -4370,16 +4367,16 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E85" s="6" t="n">
         <f aca="false">E76+E84</f>
-        <v>361.4</v>
+        <v>363.4</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B87" s="8"/>
       <c r="C87" s="8"/>
@@ -4395,7 +4392,7 @@
     </row>
     <row r="88" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B88" s="9" t="s">
         <v>19</v>
@@ -4411,33 +4408,33 @@
         <v>10</v>
       </c>
       <c r="F88" s="25" t="s">
+        <v>293</v>
+      </c>
+      <c r="G88" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H88" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I88" s="14" t="s">
         <v>294</v>
-      </c>
-      <c r="G88" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H88" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="I88" s="14" t="s">
-        <v>295</v>
       </c>
       <c r="J88" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K88" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="L88" s="9" t="s">
         <v>296</v>
-      </c>
-      <c r="L88" s="9" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="B89" s="9" t="s">
         <v>298</v>
-      </c>
-      <c r="B89" s="9" t="s">
-        <v>299</v>
       </c>
       <c r="C89" s="10" t="n">
         <v>2</v>
@@ -4450,7 +4447,7 @@
         <v>6</v>
       </c>
       <c r="F89" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G89" s="9" t="s">
         <v>21</v>
@@ -4459,24 +4456,24 @@
         <v>22</v>
       </c>
       <c r="I89" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J89" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K89" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="L89" s="9" t="s">
         <v>301</v>
-      </c>
-      <c r="L89" s="9" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="B90" s="9" t="s">
         <v>303</v>
-      </c>
-      <c r="B90" s="9" t="s">
-        <v>304</v>
       </c>
       <c r="C90" s="10" t="n">
         <v>1</v>
@@ -4489,7 +4486,7 @@
         <v>5</v>
       </c>
       <c r="F90" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G90" s="9" t="s">
         <v>21</v>
@@ -4498,21 +4495,21 @@
         <v>22</v>
       </c>
       <c r="I90" s="14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J90" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K90" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="L90" s="9" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="9" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B91" s="9" t="s">
         <v>19</v>
@@ -4528,7 +4525,7 @@
         <v>1.5</v>
       </c>
       <c r="F91" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G91" s="9" t="s">
         <v>21</v>
@@ -4537,24 +4534,24 @@
         <v>22</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J91" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K91" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="L91" s="9" t="s">
         <v>309</v>
-      </c>
-      <c r="L91" s="9" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="9" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C92" s="10" t="n">
         <v>1</v>
@@ -4567,33 +4564,33 @@
         <v>0</v>
       </c>
       <c r="F92" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="G92" s="9" t="s">
         <v>312</v>
       </c>
-      <c r="G92" s="9" t="s">
+      <c r="H92" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="I92" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="H92" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="I92" s="14" t="s">
+      <c r="J92" s="15" t="s">
         <v>314</v>
       </c>
-      <c r="J92" s="15" t="s">
+      <c r="K92" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="K92" s="9" t="s">
+      <c r="L92" s="9" t="s">
         <v>316</v>
-      </c>
-      <c r="L92" s="9" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="9" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B93" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C93" s="10" t="n">
         <v>1</v>
@@ -4606,24 +4603,24 @@
         <v>2</v>
       </c>
       <c r="F93" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="G93" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="G93" s="9" t="s">
-        <v>320</v>
       </c>
       <c r="H93" s="17"/>
       <c r="I93" s="17"/>
       <c r="J93" s="15"/>
       <c r="K93" s="9" t="s">
+        <v>320</v>
+      </c>
+      <c r="L93" s="9" t="s">
         <v>321</v>
-      </c>
-      <c r="L93" s="9" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B94" s="20"/>
       <c r="C94" s="20"/>
@@ -4642,16 +4639,16 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E95" s="6" t="n">
         <f aca="false">E76+E94</f>
-        <v>352.9</v>
+        <v>354.9</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="8" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
@@ -4667,10 +4664,10 @@
     </row>
     <row r="98" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="9" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C98" s="10" t="n">
         <v>1</v>
@@ -4683,27 +4680,27 @@
         <v>18</v>
       </c>
       <c r="F98" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H98" s="17"/>
       <c r="I98" s="17"/>
       <c r="J98" s="15"/>
       <c r="K98" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="L98" s="9" t="s">
         <v>328</v>
-      </c>
-      <c r="L98" s="9" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="9" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C99" s="10" t="n">
         <v>1</v>
@@ -4716,27 +4713,27 @@
         <v>25</v>
       </c>
       <c r="F99" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G99" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H99" s="17"/>
       <c r="I99" s="17"/>
       <c r="J99" s="15"/>
       <c r="K99" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="L99" s="9" t="s">
         <v>331</v>
-      </c>
-      <c r="L99" s="9" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="9" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B100" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C100" s="10" t="n">
         <v>1</v>
@@ -4749,27 +4746,27 @@
         <v>7</v>
       </c>
       <c r="F100" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H100" s="17"/>
       <c r="I100" s="17"/>
       <c r="J100" s="15"/>
       <c r="K100" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="L100" s="9" t="s">
         <v>334</v>
-      </c>
-      <c r="L100" s="9" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="9" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C101" s="10" t="n">
         <v>1</v>
@@ -4782,31 +4779,31 @@
         <v>38</v>
       </c>
       <c r="F101" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G101" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="H101" s="14" t="s">
         <v>337</v>
-      </c>
-      <c r="H101" s="14" t="s">
-        <v>338</v>
       </c>
       <c r="I101" s="17"/>
       <c r="J101" s="15" t="s">
+        <v>338</v>
+      </c>
+      <c r="K101" s="9" t="s">
         <v>339</v>
       </c>
-      <c r="K101" s="9" t="s">
+      <c r="L101" s="9" t="s">
         <v>340</v>
-      </c>
-      <c r="L101" s="9" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="9" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B102" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C102" s="10" t="n">
         <v>1</v>
@@ -4819,31 +4816,31 @@
         <v>15</v>
       </c>
       <c r="F102" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G102" s="9" t="s">
         <v>21</v>
       </c>
       <c r="H102" s="14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I102" s="17"/>
       <c r="J102" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K102" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="L102" s="9" t="s">
         <v>344</v>
-      </c>
-      <c r="L102" s="9" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B103" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C103" s="10" t="n">
         <v>1</v>
@@ -4856,27 +4853,27 @@
         <v>25</v>
       </c>
       <c r="F103" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G103" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H103" s="17"/>
       <c r="I103" s="17"/>
       <c r="J103" s="15"/>
       <c r="K103" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="L103" s="9" t="s">
         <v>347</v>
-      </c>
-      <c r="L103" s="9" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="9" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B104" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C104" s="10" t="n">
         <v>1</v>
@@ -4889,24 +4886,24 @@
         <v>4.3</v>
       </c>
       <c r="F104" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H104" s="17"/>
       <c r="I104" s="17"/>
       <c r="J104" s="15"/>
       <c r="K104" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="L104" s="9" t="s">
         <v>350</v>
-      </c>
-      <c r="L104" s="9" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="19" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B105" s="20"/>
       <c r="C105" s="20"/>
@@ -4925,16 +4922,16 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E106" s="6" t="n">
         <f aca="false">E76-E105</f>
-        <v>196.1</v>
+        <v>198.1</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B108" s="8"/>
       <c r="C108" s="8"/>
@@ -4950,7 +4947,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="27" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B109" s="27"/>
       <c r="C109" s="27"/>
@@ -4966,7 +4963,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="27" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B110" s="27"/>
       <c r="C110" s="27"/>
@@ -4982,7 +4979,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="27" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B111" s="27"/>
       <c r="C111" s="27"/>
@@ -4998,7 +4995,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B113" s="8"/>
       <c r="C113" s="8"/>
@@ -5014,7 +5011,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="28" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B114" s="28"/>
       <c r="C114" s="28"/>
@@ -5030,7 +5027,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="28" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B115" s="28"/>
       <c r="C115" s="28"/>
@@ -5046,7 +5043,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="28" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B116" s="28"/>
       <c r="C116" s="28"/>
@@ -5062,7 +5059,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="28" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B117" s="28"/>
       <c r="C117" s="28"/>
@@ -5078,7 +5075,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="28" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B118" s="28"/>
       <c r="C118" s="28"/>
@@ -5094,7 +5091,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="28" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B119" s="28"/>
       <c r="C119" s="28"/>
@@ -5151,7 +5148,7 @@
     <hyperlink ref="I14" r:id="rId12" display="AliExpress search: GT2 idler 20T 5 mm"/>
     <hyperlink ref="H15" r:id="rId13" display="AliExpress: 24 V adapter (pick 10A, AU plug)"/>
     <hyperlink ref="I15" r:id="rId14" display="AliExpress search: 24V 10A power supply"/>
-    <hyperlink ref="H16" r:id="rId15" display="AliExpress: AMASS XT60 (smallest pack)"/>
+    <hyperlink ref="H16" r:id="rId15" display="AliExpress: XT60H (10 pcs = 5 pairs)"/>
     <hyperlink ref="I16" r:id="rId16" display="AliExpress search: XT60 pair"/>
     <hyperlink ref="H17" r:id="rId17" display="AliExpress – DAZ's link"/>
     <hyperlink ref="I17" r:id="rId18" display="AliExpress search: 16 mm cross clamp"/>

</xml_diff>